<commit_message>
Update source files, scripts, and outputs
</commit_message>
<xml_diff>
--- a/docs/MP2027/FY2027配賦額一覧 (2025.12.29).xlsx
+++ b/docs/MP2027/FY2027配賦額一覧 (2025.12.29).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\fstvn01\Data\10_Production Engineering Department(製造技術部)\02.製造技術課\PE Dept\20. OTHERS-その他\FILE cần lưu\PA\Tổng hợp\MP2027\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sandbox\MP2027\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA45185E-E29C-407C-A1F3-A78DC31D4AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5B7768-A5C0-47B9-B0F2-0AC343B9B361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3650" yWindow="10690" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="配賦額一覧" sheetId="1" state="hidden" r:id="rId1"/>
@@ -39,9 +39,9 @@
     <definedName name="NO.2_Factory_" localSheetId="1">[3]SALＡRY!#REF!</definedName>
     <definedName name="NO.2_Factory_" localSheetId="0">[3]SALＡRY!#REF!</definedName>
     <definedName name="NO.2_Factory_">[3]SALＡRY!#REF!</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">FY2027配賦額一覧!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">FY2027配賦額一覧!$B$4:$J$71</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">配賦額一覧!$A$1:$J$81</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">FY2027配賦額一覧!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="216">
   <si>
     <t>配布元
 Phòng phân bổ</t>
@@ -1335,6 +1335,11 @@
       </rPr>
       <t>(Bao gồm cả nhân viên biệt phái)</t>
     </r>
+  </si>
+  <si>
+    <t>入社月
+入社月の翌月
+11月</t>
   </si>
 </sst>
 </file>
@@ -5072,37 +5077,37 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="41" fillId="26" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1804">
@@ -5131,6 +5136,7 @@
     <cellStyle name="Accent5 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
     <cellStyle name="Accent6 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
     <cellStyle name="Bad 2" xfId="27" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
     <cellStyle name="Calculation 2" xfId="28" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
     <cellStyle name="Calculation 2 10" xfId="793" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
     <cellStyle name="Calculation 2 11" xfId="806" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
@@ -5420,7 +5426,6 @@
     <cellStyle name="Calculation 2 8" xfId="416" xr:uid="{00000000-0005-0000-0000-000037010000}"/>
     <cellStyle name="Calculation 2 9" xfId="451" xr:uid="{00000000-0005-0000-0000-000038010000}"/>
     <cellStyle name="Check Cell 2" xfId="29" xr:uid="{00000000-0005-0000-0000-000039010000}"/>
-    <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Comma [0] 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00003B010000}"/>
     <cellStyle name="Comma [0] 3" xfId="31" xr:uid="{00000000-0005-0000-0000-00003C010000}"/>
     <cellStyle name="Comma 10" xfId="32" xr:uid="{00000000-0005-0000-0000-00003D010000}"/>
@@ -5434,13 +5439,13 @@
     <cellStyle name="Comma 7" xfId="40" xr:uid="{00000000-0005-0000-0000-000045010000}"/>
     <cellStyle name="Comma 8" xfId="41" xr:uid="{00000000-0005-0000-0000-000046010000}"/>
     <cellStyle name="Comma 9" xfId="42" xr:uid="{00000000-0005-0000-0000-000047010000}"/>
+    <cellStyle name="Dấu phẩy [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Explanatory Text 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000048010000}"/>
     <cellStyle name="Good 2" xfId="44" xr:uid="{00000000-0005-0000-0000-000049010000}"/>
     <cellStyle name="Heading 1 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00004A010000}"/>
     <cellStyle name="Heading 2 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00004B010000}"/>
     <cellStyle name="Heading 3 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00004C010000}"/>
     <cellStyle name="Heading 4 2" xfId="48" xr:uid="{00000000-0005-0000-0000-00004D010000}"/>
-    <cellStyle name="Hyperlink" xfId="92" builtinId="8"/>
     <cellStyle name="Input 2" xfId="49" xr:uid="{00000000-0005-0000-0000-00004F010000}"/>
     <cellStyle name="Input 2 10" xfId="1020" xr:uid="{00000000-0005-0000-0000-000050010000}"/>
     <cellStyle name="Input 2 11" xfId="1171" xr:uid="{00000000-0005-0000-0000-000051010000}"/>
@@ -5731,7 +5736,6 @@
     <cellStyle name="Input 2 9" xfId="432" xr:uid="{00000000-0005-0000-0000-00006E020000}"/>
     <cellStyle name="Linked Cell 2" xfId="50" xr:uid="{00000000-0005-0000-0000-00006F020000}"/>
     <cellStyle name="Neutral 2" xfId="51" xr:uid="{00000000-0005-0000-0000-000070020000}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal - Style1" xfId="52" xr:uid="{00000000-0005-0000-0000-000072020000}"/>
     <cellStyle name="Normal 10" xfId="53" xr:uid="{00000000-0005-0000-0000-000073020000}"/>
     <cellStyle name="Normal 11" xfId="54" xr:uid="{00000000-0005-0000-0000-000074020000}"/>
@@ -6425,6 +6429,7 @@
     <cellStyle name="Output 2 9" xfId="410" xr:uid="{00000000-0005-0000-0000-000024050000}"/>
     <cellStyle name="Percent 2" xfId="72" xr:uid="{00000000-0005-0000-0000-000025050000}"/>
     <cellStyle name="Percent 2 2" xfId="124" xr:uid="{00000000-0005-0000-0000-000026050000}"/>
+    <cellStyle name="Siêu kết nối" xfId="92" builtinId="8"/>
     <cellStyle name="Title 2" xfId="73" xr:uid="{00000000-0005-0000-0000-000027050000}"/>
     <cellStyle name="Total 2" xfId="74" xr:uid="{00000000-0005-0000-0000-000028050000}"/>
     <cellStyle name="Total 2 10" xfId="889" xr:uid="{00000000-0005-0000-0000-000029050000}"/>
@@ -7326,22 +7331,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K85"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13" style="3" customWidth="1"/>
-    <col min="2" max="2" width="26.36328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="13" style="3" customWidth="1"/>
-    <col min="5" max="6" width="15.26953125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.36328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="13.7265625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" style="2" customWidth="1"/>
+    <col min="5" max="6" width="15.28515625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="2" customWidth="1"/>
     <col min="10" max="10" width="110" style="2" customWidth="1"/>
-    <col min="11" max="11" width="10.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.5">
+    <row r="1" spans="1:10" ht="18">
       <c r="A1" s="1" t="s">
         <v>148</v>
       </c>
@@ -7394,8 +7399,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="45.65" customHeight="1">
-      <c r="A5" s="92" t="s">
+    <row r="5" spans="1:10" ht="45.6" customHeight="1">
+      <c r="A5" s="90" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="21" t="s">
@@ -7521,19 +7526,19 @@
       <c r="B9" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="93" t="s">
+      <c r="C9" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="93">
+      <c r="D9" s="96">
         <v>5005246288</v>
       </c>
-      <c r="E9" s="93">
+      <c r="E9" s="96">
         <v>6005126423</v>
       </c>
-      <c r="F9" s="93">
+      <c r="F9" s="96">
         <v>6005246544</v>
       </c>
-      <c r="G9" s="93" t="s">
+      <c r="G9" s="96" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="38">
@@ -7549,11 +7554,11 @@
     <row r="10" spans="1:10" ht="31.5" customHeight="1">
       <c r="A10" s="89"/>
       <c r="B10" s="95"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
+      <c r="C10" s="96"/>
+      <c r="D10" s="96"/>
+      <c r="E10" s="96"/>
+      <c r="F10" s="96"/>
+      <c r="G10" s="96"/>
       <c r="H10" s="38">
         <v>9100</v>
       </c>
@@ -7625,7 +7630,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="33" customHeight="1">
-      <c r="A13" s="96"/>
+      <c r="A13" s="99"/>
       <c r="B13" s="26" t="s">
         <v>28</v>
       </c>
@@ -7745,7 +7750,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="34.5" customHeight="1">
-      <c r="A17" s="97"/>
+      <c r="A17" s="100"/>
       <c r="B17" s="32" t="s">
         <v>41</v>
       </c>
@@ -7775,7 +7780,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="36.75" customHeight="1">
-      <c r="A18" s="92" t="s">
+      <c r="A18" s="90" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="21" t="s">
@@ -7802,7 +7807,7 @@
       <c r="I18" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="J18" s="90" t="s">
+      <c r="J18" s="97" t="s">
         <v>176</v>
       </c>
       <c r="K18" s="10"/>
@@ -7833,7 +7838,7 @@
       <c r="I19" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="91"/>
+      <c r="J19" s="98"/>
       <c r="K19" s="10" t="s">
         <v>187</v>
       </c>
@@ -7864,7 +7869,7 @@
       <c r="I20" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="J20" s="91"/>
+      <c r="J20" s="98"/>
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="85.5" customHeight="1">
@@ -9064,7 +9069,7 @@
       </c>
       <c r="K60" s="57"/>
     </row>
-    <row r="61" spans="1:11" ht="92.15" customHeight="1">
+    <row r="61" spans="1:11" ht="92.1" customHeight="1">
       <c r="A61" s="89"/>
       <c r="B61" s="42" t="s">
         <v>110</v>
@@ -9219,7 +9224,7 @@
       </c>
       <c r="K65" s="10"/>
     </row>
-    <row r="66" spans="1:11" ht="138.65" customHeight="1">
+    <row r="66" spans="1:11" ht="138.6" customHeight="1">
       <c r="A66" s="89"/>
       <c r="B66" s="42" t="s">
         <v>117</v>
@@ -9250,7 +9255,7 @@
       </c>
       <c r="K66" s="10"/>
     </row>
-    <row r="67" spans="1:11" ht="314.14999999999998" customHeight="1">
+    <row r="67" spans="1:11" ht="314.10000000000002" customHeight="1">
       <c r="A67" s="89"/>
       <c r="B67" s="42" t="s">
         <v>119</v>
@@ -9693,22 +9698,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13" style="3" customWidth="1"/>
-    <col min="2" max="2" width="35.26953125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.7265625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="13" style="3" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.36328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.26953125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="113.36328125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="113.42578125" style="2" customWidth="1"/>
     <col min="11" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.5">
+    <row r="1" spans="1:10" ht="18">
       <c r="A1" s="1" t="s">
         <v>189</v>
       </c>
@@ -9761,8 +9766,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="58" customFormat="1" ht="38.5" customHeight="1">
-      <c r="A5" s="98" t="s">
+    <row r="5" spans="1:10" s="58" customFormat="1" ht="38.450000000000003" customHeight="1">
+      <c r="A5" s="91" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="21" t="s">
@@ -9794,7 +9799,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A6" s="99"/>
+      <c r="A6" s="92"/>
       <c r="B6" s="26" t="s">
         <v>16</v>
       </c>
@@ -9824,7 +9829,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A7" s="99"/>
+      <c r="A7" s="92"/>
       <c r="B7" s="26" t="s">
         <v>18</v>
       </c>
@@ -9854,7 +9859,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A8" s="99"/>
+      <c r="A8" s="92"/>
       <c r="B8" s="30" t="s">
         <v>21</v>
       </c>
@@ -9884,23 +9889,23 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A9" s="99"/>
+      <c r="A9" s="92"/>
       <c r="B9" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="93" t="s">
+      <c r="C9" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="93">
+      <c r="D9" s="96">
         <v>5005246288</v>
       </c>
-      <c r="E9" s="93">
+      <c r="E9" s="96">
         <v>6005126423</v>
       </c>
-      <c r="F9" s="93">
+      <c r="F9" s="96">
         <v>6005246544</v>
       </c>
-      <c r="G9" s="93" t="s">
+      <c r="G9" s="96" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="38">
@@ -9914,13 +9919,13 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A10" s="99"/>
+      <c r="A10" s="92"/>
       <c r="B10" s="95"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
+      <c r="C10" s="96"/>
+      <c r="D10" s="96"/>
+      <c r="E10" s="96"/>
+      <c r="F10" s="96"/>
+      <c r="G10" s="96"/>
       <c r="H10" s="38">
         <v>9100</v>
       </c>
@@ -9932,7 +9937,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A11" s="99"/>
+      <c r="A11" s="92"/>
       <c r="B11" s="26" t="s">
         <v>149</v>
       </c>
@@ -9962,7 +9967,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A12" s="99"/>
+      <c r="A12" s="92"/>
       <c r="B12" s="26" t="s">
         <v>150</v>
       </c>
@@ -9992,7 +9997,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A13" s="99"/>
+      <c r="A13" s="92"/>
       <c r="B13" s="26" t="s">
         <v>28</v>
       </c>
@@ -10022,7 +10027,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" s="58" customFormat="1" ht="83.25" customHeight="1">
-      <c r="A14" s="99"/>
+      <c r="A14" s="92"/>
       <c r="B14" s="42" t="s">
         <v>32</v>
       </c>
@@ -10052,7 +10057,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A15" s="99"/>
+      <c r="A15" s="92"/>
       <c r="B15" s="42" t="s">
         <v>35</v>
       </c>
@@ -10082,7 +10087,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" s="58" customFormat="1" ht="84" customHeight="1">
-      <c r="A16" s="99"/>
+      <c r="A16" s="92"/>
       <c r="B16" s="42" t="s">
         <v>39</v>
       </c>
@@ -10112,7 +10117,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A17" s="100"/>
+      <c r="A17" s="93"/>
       <c r="B17" s="32" t="s">
         <v>41</v>
       </c>
@@ -10142,7 +10147,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A18" s="98" t="s">
+      <c r="A18" s="91" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="21" t="s">
@@ -10169,12 +10174,12 @@
       <c r="I18" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="J18" s="92" t="s">
+      <c r="J18" s="90" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A19" s="99"/>
+      <c r="A19" s="92"/>
       <c r="B19" s="26" t="s">
         <v>51</v>
       </c>
@@ -10202,7 +10207,7 @@
       <c r="J19" s="89"/>
     </row>
     <row r="20" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A20" s="99"/>
+      <c r="A20" s="92"/>
       <c r="B20" s="26" t="s">
         <v>52</v>
       </c>
@@ -10230,7 +10235,7 @@
       <c r="J20" s="89"/>
     </row>
     <row r="21" spans="1:10" ht="85.5" customHeight="1">
-      <c r="A21" s="99"/>
+      <c r="A21" s="92"/>
       <c r="B21" s="26" t="s">
         <v>53</v>
       </c>
@@ -10258,7 +10263,7 @@
       <c r="J21" s="89"/>
     </row>
     <row r="22" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A22" s="99"/>
+      <c r="A22" s="92"/>
       <c r="B22" s="26" t="s">
         <v>55</v>
       </c>
@@ -10288,7 +10293,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A23" s="99"/>
+      <c r="A23" s="92"/>
       <c r="B23" s="26" t="s">
         <v>60</v>
       </c>
@@ -10318,7 +10323,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A24" s="99"/>
+      <c r="A24" s="92"/>
       <c r="B24" s="26" t="s">
         <v>195</v>
       </c>
@@ -10346,7 +10351,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A25" s="99"/>
+      <c r="A25" s="92"/>
       <c r="B25" s="26" t="s">
         <v>63</v>
       </c>
@@ -10374,7 +10379,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="31.5" customHeight="1">
-      <c r="A26" s="99"/>
+      <c r="A26" s="92"/>
       <c r="B26" s="42" t="s">
         <v>197</v>
       </c>
@@ -10402,7 +10407,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A27" s="99"/>
+      <c r="A27" s="92"/>
       <c r="B27" s="30" t="s">
         <v>66</v>
       </c>
@@ -10430,7 +10435,7 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A28" s="99"/>
+      <c r="A28" s="92"/>
       <c r="B28" s="30" t="s">
         <v>68</v>
       </c>
@@ -10458,7 +10463,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="46.5" customHeight="1">
-      <c r="A29" s="99"/>
+      <c r="A29" s="92"/>
       <c r="B29" s="26" t="s">
         <v>69</v>
       </c>
@@ -10488,7 +10493,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="46.5" customHeight="1">
-      <c r="A30" s="99"/>
+      <c r="A30" s="92"/>
       <c r="B30" s="26" t="s">
         <v>72</v>
       </c>
@@ -10516,7 +10521,7 @@
       <c r="J30" s="89"/>
     </row>
     <row r="31" spans="1:10" s="58" customFormat="1" ht="66" customHeight="1">
-      <c r="A31" s="99"/>
+      <c r="A31" s="92"/>
       <c r="B31" s="42" t="s">
         <v>73</v>
       </c>
@@ -10533,7 +10538,7 @@
         <v>6005146541</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>154</v>
+        <v>215</v>
       </c>
       <c r="H31" s="59">
         <v>760</v>
@@ -10546,7 +10551,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="43.5" customHeight="1">
-      <c r="A32" s="99"/>
+      <c r="A32" s="92"/>
       <c r="B32" s="26" t="s">
         <v>74</v>
       </c>
@@ -10576,7 +10581,7 @@
       </c>
     </row>
     <row r="33" spans="1:10" ht="40.5" customHeight="1">
-      <c r="A33" s="99"/>
+      <c r="A33" s="92"/>
       <c r="B33" s="26" t="s">
         <v>77</v>
       </c>
@@ -10606,7 +10611,7 @@
       </c>
     </row>
     <row r="34" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A34" s="99"/>
+      <c r="A34" s="92"/>
       <c r="B34" s="26" t="s">
         <v>79</v>
       </c>
@@ -10636,7 +10641,7 @@
       </c>
     </row>
     <row r="35" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A35" s="99"/>
+      <c r="A35" s="92"/>
       <c r="B35" s="26" t="s">
         <v>80</v>
       </c>
@@ -10666,7 +10671,7 @@
       </c>
     </row>
     <row r="36" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A36" s="99"/>
+      <c r="A36" s="92"/>
       <c r="B36" s="26" t="s">
         <v>153</v>
       </c>
@@ -10696,7 +10701,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A37" s="99"/>
+      <c r="A37" s="92"/>
       <c r="B37" s="26" t="s">
         <v>82</v>
       </c>
@@ -10726,7 +10731,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A38" s="99"/>
+      <c r="A38" s="92"/>
       <c r="B38" s="26" t="s">
         <v>83</v>
       </c>
@@ -10756,7 +10761,7 @@
       </c>
     </row>
     <row r="39" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A39" s="99"/>
+      <c r="A39" s="92"/>
       <c r="B39" s="26" t="s">
         <v>84</v>
       </c>
@@ -10786,7 +10791,7 @@
       </c>
     </row>
     <row r="40" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A40" s="99"/>
+      <c r="A40" s="92"/>
       <c r="B40" s="26" t="s">
         <v>163</v>
       </c>
@@ -10816,7 +10821,7 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A41" s="99"/>
+      <c r="A41" s="92"/>
       <c r="B41" s="26" t="s">
         <v>85</v>
       </c>
@@ -10846,7 +10851,7 @@
       </c>
     </row>
     <row r="42" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A42" s="99"/>
+      <c r="A42" s="92"/>
       <c r="B42" s="26" t="s">
         <v>86</v>
       </c>
@@ -10876,7 +10881,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A43" s="99"/>
+      <c r="A43" s="92"/>
       <c r="B43" s="26" t="s">
         <v>88</v>
       </c>
@@ -10906,7 +10911,7 @@
       </c>
     </row>
     <row r="44" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A44" s="99"/>
+      <c r="A44" s="92"/>
       <c r="B44" s="26" t="s">
         <v>90</v>
       </c>
@@ -10936,7 +10941,7 @@
       </c>
     </row>
     <row r="45" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A45" s="99"/>
+      <c r="A45" s="92"/>
       <c r="B45" s="42" t="s">
         <v>168</v>
       </c>
@@ -10966,7 +10971,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" ht="42" customHeight="1">
-      <c r="A46" s="99"/>
+      <c r="A46" s="92"/>
       <c r="B46" s="26" t="s">
         <v>173</v>
       </c>
@@ -10996,7 +11001,7 @@
       </c>
     </row>
     <row r="47" spans="1:10" ht="99.75" customHeight="1">
-      <c r="A47" s="99"/>
+      <c r="A47" s="92"/>
       <c r="B47" s="42" t="s">
         <v>174</v>
       </c>
@@ -11026,7 +11031,7 @@
       </c>
     </row>
     <row r="48" spans="1:10" ht="42" customHeight="1">
-      <c r="A48" s="99"/>
+      <c r="A48" s="92"/>
       <c r="B48" s="26" t="s">
         <v>91</v>
       </c>
@@ -11056,7 +11061,7 @@
       </c>
     </row>
     <row r="49" spans="1:10" ht="42" customHeight="1">
-      <c r="A49" s="99"/>
+      <c r="A49" s="92"/>
       <c r="B49" s="26" t="s">
         <v>92</v>
       </c>
@@ -11086,7 +11091,7 @@
       </c>
     </row>
     <row r="50" spans="1:10" ht="42" customHeight="1">
-      <c r="A50" s="99"/>
+      <c r="A50" s="92"/>
       <c r="B50" s="26" t="s">
         <v>94</v>
       </c>
@@ -11116,7 +11121,7 @@
       </c>
     </row>
     <row r="51" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A51" s="99"/>
+      <c r="A51" s="92"/>
       <c r="B51" s="26" t="s">
         <v>95</v>
       </c>
@@ -11146,7 +11151,7 @@
       </c>
     </row>
     <row r="52" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A52" s="99"/>
+      <c r="A52" s="92"/>
       <c r="B52" s="26" t="s">
         <v>96</v>
       </c>
@@ -11176,7 +11181,7 @@
       </c>
     </row>
     <row r="53" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A53" s="99"/>
+      <c r="A53" s="92"/>
       <c r="B53" s="26" t="s">
         <v>97</v>
       </c>
@@ -11206,7 +11211,7 @@
       </c>
     </row>
     <row r="54" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A54" s="99"/>
+      <c r="A54" s="92"/>
       <c r="B54" s="26" t="s">
         <v>99</v>
       </c>
@@ -11236,7 +11241,7 @@
       </c>
     </row>
     <row r="55" spans="1:10" s="58" customFormat="1" ht="85.5" customHeight="1">
-      <c r="A55" s="99"/>
+      <c r="A55" s="92"/>
       <c r="B55" s="42" t="s">
         <v>101</v>
       </c>
@@ -11266,7 +11271,7 @@
       </c>
     </row>
     <row r="56" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A56" s="99"/>
+      <c r="A56" s="92"/>
       <c r="B56" s="42" t="s">
         <v>102</v>
       </c>
@@ -11296,7 +11301,7 @@
       </c>
     </row>
     <row r="57" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A57" s="99"/>
+      <c r="A57" s="92"/>
       <c r="B57" s="42" t="s">
         <v>104</v>
       </c>
@@ -11326,7 +11331,7 @@
       </c>
     </row>
     <row r="58" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A58" s="99"/>
+      <c r="A58" s="92"/>
       <c r="B58" s="42" t="s">
         <v>105</v>
       </c>
@@ -11356,7 +11361,7 @@
       </c>
     </row>
     <row r="59" spans="1:10" s="65" customFormat="1" ht="54.75" customHeight="1">
-      <c r="A59" s="99"/>
+      <c r="A59" s="92"/>
       <c r="B59" s="56" t="s">
         <v>106</v>
       </c>
@@ -11386,7 +11391,7 @@
       </c>
     </row>
     <row r="60" spans="1:10" s="71" customFormat="1" ht="60" customHeight="1">
-      <c r="A60" s="99"/>
+      <c r="A60" s="92"/>
       <c r="B60" s="42" t="s">
         <v>210</v>
       </c>
@@ -11416,7 +11421,7 @@
       </c>
     </row>
     <row r="61" spans="1:10" ht="114" customHeight="1">
-      <c r="A61" s="99"/>
+      <c r="A61" s="92"/>
       <c r="B61" s="42" t="s">
         <v>107</v>
       </c>
@@ -11446,7 +11451,7 @@
       </c>
     </row>
     <row r="62" spans="1:10" ht="139.15" customHeight="1">
-      <c r="A62" s="99"/>
+      <c r="A62" s="92"/>
       <c r="B62" s="42" t="s">
         <v>171</v>
       </c>
@@ -11476,7 +11481,7 @@
       </c>
     </row>
     <row r="63" spans="1:10" s="58" customFormat="1" ht="93.75" customHeight="1">
-      <c r="A63" s="99"/>
+      <c r="A63" s="92"/>
       <c r="B63" s="42" t="s">
         <v>109</v>
       </c>
@@ -11506,7 +11511,7 @@
       </c>
     </row>
     <row r="64" spans="1:10" ht="135" customHeight="1">
-      <c r="A64" s="99"/>
+      <c r="A64" s="92"/>
       <c r="B64" s="42" t="s">
         <v>110</v>
       </c>
@@ -11536,7 +11541,7 @@
       </c>
     </row>
     <row r="65" spans="1:10" ht="138" customHeight="1">
-      <c r="A65" s="99"/>
+      <c r="A65" s="92"/>
       <c r="B65" s="41" t="s">
         <v>111</v>
       </c>
@@ -11566,7 +11571,7 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="96" customHeight="1">
-      <c r="A66" s="99"/>
+      <c r="A66" s="92"/>
       <c r="B66" s="41" t="s">
         <v>113</v>
       </c>
@@ -11596,7 +11601,7 @@
       </c>
     </row>
     <row r="67" spans="1:10" ht="95.25" customHeight="1">
-      <c r="A67" s="99"/>
+      <c r="A67" s="92"/>
       <c r="B67" s="42" t="s">
         <v>147</v>
       </c>
@@ -11626,7 +11631,7 @@
       </c>
     </row>
     <row r="68" spans="1:10" s="65" customFormat="1" ht="60" customHeight="1">
-      <c r="A68" s="99"/>
+      <c r="A68" s="92"/>
       <c r="B68" s="56" t="s">
         <v>116</v>
       </c>
@@ -11656,7 +11661,7 @@
       </c>
     </row>
     <row r="69" spans="1:10" ht="163.5" customHeight="1">
-      <c r="A69" s="99"/>
+      <c r="A69" s="92"/>
       <c r="B69" s="42" t="s">
         <v>117</v>
       </c>
@@ -11686,7 +11691,7 @@
       </c>
     </row>
     <row r="70" spans="1:10" ht="334.5" customHeight="1">
-      <c r="A70" s="99"/>
+      <c r="A70" s="92"/>
       <c r="B70" s="42" t="s">
         <v>119</v>
       </c>
@@ -11716,7 +11721,7 @@
       </c>
     </row>
     <row r="71" spans="1:10" s="71" customFormat="1" ht="150" customHeight="1">
-      <c r="A71" s="100"/>
+      <c r="A71" s="93"/>
       <c r="B71" s="80" t="s">
         <v>211</v>
       </c>
@@ -11844,17 +11849,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Tài liệu" ma:contentTypeID="0x010100DB24EDB465323845A68F49B67C0FBEEF" ma:contentTypeVersion="17" ma:contentTypeDescription="Tạo tài liệu mới." ma:contentTypeScope="" ma:versionID="23f0dc0ab5ad78d6e6291fdb2fe26642">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3666f02-6a17-4b93-8e4f-4f8c851bed15" xmlns:ns3="a67f3886-f84f-4ade-a9df-8a61292dc710" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c7e7713e468ce5fe561a860222c69c2e" ns2:_="" ns3:_="">
     <xsd:import namespace="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
@@ -12031,32 +12025,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64BA0B11-CE17-4EF2-86D1-BF1E203BBB04}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="a67f3886-f84f-4ade-a9df-8a61292dc710"/>
-    <ds:schemaRef ds:uri="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC0FACC-084E-4CA6-AB6A-54805DEE3D3C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC458EFE-CB2F-4B14-8A64-8A5C4D5C5CBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12073,4 +12053,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC0FACC-084E-4CA6-AB6A-54805DEE3D3C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64BA0B11-CE17-4EF2-86D1-BF1E203BBB04}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="a67f3886-f84f-4ade-a9df-8a61292dc710"/>
+    <ds:schemaRef ds:uri="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Remove generated data from pushed changes
</commit_message>
<xml_diff>
--- a/docs/MP2027/FY2027配賦額一覧 (2025.12.29).xlsx
+++ b/docs/MP2027/FY2027配賦額一覧 (2025.12.29).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sandbox\MP2027\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\fstvn01\Data\10_Production Engineering Department(製造技術部)\02.製造技術課\PE Dept\20. OTHERS-その他\FILE cần lưu\PA\Tổng hợp\MP2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5B7768-A5C0-47B9-B0F2-0AC343B9B361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA45185E-E29C-407C-A1F3-A78DC31D4AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3650" yWindow="10690" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="配賦額一覧" sheetId="1" state="hidden" r:id="rId1"/>
@@ -39,9 +39,9 @@
     <definedName name="NO.2_Factory_" localSheetId="1">[3]SALＡRY!#REF!</definedName>
     <definedName name="NO.2_Factory_" localSheetId="0">[3]SALＡRY!#REF!</definedName>
     <definedName name="NO.2_Factory_">[3]SALＡRY!#REF!</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">FY2027配賦額一覧!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">FY2027配賦額一覧!$B$4:$J$71</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">配賦額一覧!$A$1:$J$81</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">FY2027配賦額一覧!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="215">
   <si>
     <t>配布元
 Phòng phân bổ</t>
@@ -1335,11 +1335,6 @@
       </rPr>
       <t>(Bao gồm cả nhân viên biệt phái)</t>
     </r>
-  </si>
-  <si>
-    <t>入社月
-入社月の翌月
-11月</t>
   </si>
 </sst>
 </file>
@@ -5077,6 +5072,27 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="26" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5087,27 +5103,6 @@
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="26" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1804">
@@ -5136,7 +5131,6 @@
     <cellStyle name="Accent5 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
     <cellStyle name="Accent6 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
     <cellStyle name="Bad 2" xfId="27" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
     <cellStyle name="Calculation 2" xfId="28" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
     <cellStyle name="Calculation 2 10" xfId="793" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
     <cellStyle name="Calculation 2 11" xfId="806" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
@@ -5426,6 +5420,7 @@
     <cellStyle name="Calculation 2 8" xfId="416" xr:uid="{00000000-0005-0000-0000-000037010000}"/>
     <cellStyle name="Calculation 2 9" xfId="451" xr:uid="{00000000-0005-0000-0000-000038010000}"/>
     <cellStyle name="Check Cell 2" xfId="29" xr:uid="{00000000-0005-0000-0000-000039010000}"/>
+    <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Comma [0] 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00003B010000}"/>
     <cellStyle name="Comma [0] 3" xfId="31" xr:uid="{00000000-0005-0000-0000-00003C010000}"/>
     <cellStyle name="Comma 10" xfId="32" xr:uid="{00000000-0005-0000-0000-00003D010000}"/>
@@ -5439,13 +5434,13 @@
     <cellStyle name="Comma 7" xfId="40" xr:uid="{00000000-0005-0000-0000-000045010000}"/>
     <cellStyle name="Comma 8" xfId="41" xr:uid="{00000000-0005-0000-0000-000046010000}"/>
     <cellStyle name="Comma 9" xfId="42" xr:uid="{00000000-0005-0000-0000-000047010000}"/>
-    <cellStyle name="Dấu phẩy [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Explanatory Text 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000048010000}"/>
     <cellStyle name="Good 2" xfId="44" xr:uid="{00000000-0005-0000-0000-000049010000}"/>
     <cellStyle name="Heading 1 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00004A010000}"/>
     <cellStyle name="Heading 2 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00004B010000}"/>
     <cellStyle name="Heading 3 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00004C010000}"/>
     <cellStyle name="Heading 4 2" xfId="48" xr:uid="{00000000-0005-0000-0000-00004D010000}"/>
+    <cellStyle name="Hyperlink" xfId="92" builtinId="8"/>
     <cellStyle name="Input 2" xfId="49" xr:uid="{00000000-0005-0000-0000-00004F010000}"/>
     <cellStyle name="Input 2 10" xfId="1020" xr:uid="{00000000-0005-0000-0000-000050010000}"/>
     <cellStyle name="Input 2 11" xfId="1171" xr:uid="{00000000-0005-0000-0000-000051010000}"/>
@@ -5736,6 +5731,7 @@
     <cellStyle name="Input 2 9" xfId="432" xr:uid="{00000000-0005-0000-0000-00006E020000}"/>
     <cellStyle name="Linked Cell 2" xfId="50" xr:uid="{00000000-0005-0000-0000-00006F020000}"/>
     <cellStyle name="Neutral 2" xfId="51" xr:uid="{00000000-0005-0000-0000-000070020000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal - Style1" xfId="52" xr:uid="{00000000-0005-0000-0000-000072020000}"/>
     <cellStyle name="Normal 10" xfId="53" xr:uid="{00000000-0005-0000-0000-000073020000}"/>
     <cellStyle name="Normal 11" xfId="54" xr:uid="{00000000-0005-0000-0000-000074020000}"/>
@@ -6429,7 +6425,6 @@
     <cellStyle name="Output 2 9" xfId="410" xr:uid="{00000000-0005-0000-0000-000024050000}"/>
     <cellStyle name="Percent 2" xfId="72" xr:uid="{00000000-0005-0000-0000-000025050000}"/>
     <cellStyle name="Percent 2 2" xfId="124" xr:uid="{00000000-0005-0000-0000-000026050000}"/>
-    <cellStyle name="Siêu kết nối" xfId="92" builtinId="8"/>
     <cellStyle name="Title 2" xfId="73" xr:uid="{00000000-0005-0000-0000-000027050000}"/>
     <cellStyle name="Total 2" xfId="74" xr:uid="{00000000-0005-0000-0000-000028050000}"/>
     <cellStyle name="Total 2 10" xfId="889" xr:uid="{00000000-0005-0000-0000-000029050000}"/>
@@ -7331,22 +7326,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K85"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="13" style="3" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" style="2" customWidth="1"/>
     <col min="4" max="4" width="13" style="3" customWidth="1"/>
-    <col min="5" max="6" width="15.28515625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" style="2" customWidth="1"/>
+    <col min="5" max="6" width="15.26953125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.7265625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.7265625" style="2" customWidth="1"/>
     <col min="10" max="10" width="110" style="2" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18">
+    <row r="1" spans="1:10" ht="17.5">
       <c r="A1" s="1" t="s">
         <v>148</v>
       </c>
@@ -7399,8 +7394,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="45.6" customHeight="1">
-      <c r="A5" s="90" t="s">
+    <row r="5" spans="1:10" ht="45.65" customHeight="1">
+      <c r="A5" s="92" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="21" t="s">
@@ -7526,19 +7521,19 @@
       <c r="B9" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="96" t="s">
+      <c r="C9" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="96">
+      <c r="D9" s="93">
         <v>5005246288</v>
       </c>
-      <c r="E9" s="96">
+      <c r="E9" s="93">
         <v>6005126423</v>
       </c>
-      <c r="F9" s="96">
+      <c r="F9" s="93">
         <v>6005246544</v>
       </c>
-      <c r="G9" s="96" t="s">
+      <c r="G9" s="93" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="38">
@@ -7554,11 +7549,11 @@
     <row r="10" spans="1:10" ht="31.5" customHeight="1">
       <c r="A10" s="89"/>
       <c r="B10" s="95"/>
-      <c r="C10" s="96"/>
-      <c r="D10" s="96"/>
-      <c r="E10" s="96"/>
-      <c r="F10" s="96"/>
-      <c r="G10" s="96"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
       <c r="H10" s="38">
         <v>9100</v>
       </c>
@@ -7630,7 +7625,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="33" customHeight="1">
-      <c r="A13" s="99"/>
+      <c r="A13" s="96"/>
       <c r="B13" s="26" t="s">
         <v>28</v>
       </c>
@@ -7750,7 +7745,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="34.5" customHeight="1">
-      <c r="A17" s="100"/>
+      <c r="A17" s="97"/>
       <c r="B17" s="32" t="s">
         <v>41</v>
       </c>
@@ -7780,7 +7775,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="36.75" customHeight="1">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="92" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="21" t="s">
@@ -7807,7 +7802,7 @@
       <c r="I18" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="J18" s="97" t="s">
+      <c r="J18" s="90" t="s">
         <v>176</v>
       </c>
       <c r="K18" s="10"/>
@@ -7838,7 +7833,7 @@
       <c r="I19" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="98"/>
+      <c r="J19" s="91"/>
       <c r="K19" s="10" t="s">
         <v>187</v>
       </c>
@@ -7869,7 +7864,7 @@
       <c r="I20" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="J20" s="98"/>
+      <c r="J20" s="91"/>
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="85.5" customHeight="1">
@@ -9069,7 +9064,7 @@
       </c>
       <c r="K60" s="57"/>
     </row>
-    <row r="61" spans="1:11" ht="92.1" customHeight="1">
+    <row r="61" spans="1:11" ht="92.15" customHeight="1">
       <c r="A61" s="89"/>
       <c r="B61" s="42" t="s">
         <v>110</v>
@@ -9224,7 +9219,7 @@
       </c>
       <c r="K65" s="10"/>
     </row>
-    <row r="66" spans="1:11" ht="138.6" customHeight="1">
+    <row r="66" spans="1:11" ht="138.65" customHeight="1">
       <c r="A66" s="89"/>
       <c r="B66" s="42" t="s">
         <v>117</v>
@@ -9255,7 +9250,7 @@
       </c>
       <c r="K66" s="10"/>
     </row>
-    <row r="67" spans="1:11" ht="314.10000000000002" customHeight="1">
+    <row r="67" spans="1:11" ht="314.14999999999998" customHeight="1">
       <c r="A67" s="89"/>
       <c r="B67" s="42" t="s">
         <v>119</v>
@@ -9698,22 +9693,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="13" style="3" customWidth="1"/>
-    <col min="2" max="2" width="35.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="35.26953125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.7265625" style="2" customWidth="1"/>
     <col min="4" max="4" width="13" style="3" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="113.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.26953125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.7265625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="113.36328125" style="2" customWidth="1"/>
     <col min="11" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18">
+    <row r="1" spans="1:10" ht="17.5">
       <c r="A1" s="1" t="s">
         <v>189</v>
       </c>
@@ -9766,8 +9761,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="58" customFormat="1" ht="38.450000000000003" customHeight="1">
-      <c r="A5" s="91" t="s">
+    <row r="5" spans="1:10" s="58" customFormat="1" ht="38.5" customHeight="1">
+      <c r="A5" s="98" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="21" t="s">
@@ -9799,7 +9794,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A6" s="92"/>
+      <c r="A6" s="99"/>
       <c r="B6" s="26" t="s">
         <v>16</v>
       </c>
@@ -9829,7 +9824,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A7" s="92"/>
+      <c r="A7" s="99"/>
       <c r="B7" s="26" t="s">
         <v>18</v>
       </c>
@@ -9859,7 +9854,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A8" s="92"/>
+      <c r="A8" s="99"/>
       <c r="B8" s="30" t="s">
         <v>21</v>
       </c>
@@ -9889,23 +9884,23 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A9" s="92"/>
+      <c r="A9" s="99"/>
       <c r="B9" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="96" t="s">
+      <c r="C9" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="96">
+      <c r="D9" s="93">
         <v>5005246288</v>
       </c>
-      <c r="E9" s="96">
+      <c r="E9" s="93">
         <v>6005126423</v>
       </c>
-      <c r="F9" s="96">
+      <c r="F9" s="93">
         <v>6005246544</v>
       </c>
-      <c r="G9" s="96" t="s">
+      <c r="G9" s="93" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="38">
@@ -9919,13 +9914,13 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A10" s="92"/>
+      <c r="A10" s="99"/>
       <c r="B10" s="95"/>
-      <c r="C10" s="96"/>
-      <c r="D10" s="96"/>
-      <c r="E10" s="96"/>
-      <c r="F10" s="96"/>
-      <c r="G10" s="96"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
       <c r="H10" s="38">
         <v>9100</v>
       </c>
@@ -9937,7 +9932,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A11" s="92"/>
+      <c r="A11" s="99"/>
       <c r="B11" s="26" t="s">
         <v>149</v>
       </c>
@@ -9967,7 +9962,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A12" s="92"/>
+      <c r="A12" s="99"/>
       <c r="B12" s="26" t="s">
         <v>150</v>
       </c>
@@ -9997,7 +9992,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A13" s="92"/>
+      <c r="A13" s="99"/>
       <c r="B13" s="26" t="s">
         <v>28</v>
       </c>
@@ -10027,7 +10022,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" s="58" customFormat="1" ht="83.25" customHeight="1">
-      <c r="A14" s="92"/>
+      <c r="A14" s="99"/>
       <c r="B14" s="42" t="s">
         <v>32</v>
       </c>
@@ -10057,7 +10052,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A15" s="92"/>
+      <c r="A15" s="99"/>
       <c r="B15" s="42" t="s">
         <v>35</v>
       </c>
@@ -10087,7 +10082,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" s="58" customFormat="1" ht="84" customHeight="1">
-      <c r="A16" s="92"/>
+      <c r="A16" s="99"/>
       <c r="B16" s="42" t="s">
         <v>39</v>
       </c>
@@ -10117,7 +10112,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" s="58" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A17" s="93"/>
+      <c r="A17" s="100"/>
       <c r="B17" s="32" t="s">
         <v>41</v>
       </c>
@@ -10147,7 +10142,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A18" s="91" t="s">
+      <c r="A18" s="98" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="21" t="s">
@@ -10174,12 +10169,12 @@
       <c r="I18" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="J18" s="90" t="s">
+      <c r="J18" s="92" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A19" s="92"/>
+      <c r="A19" s="99"/>
       <c r="B19" s="26" t="s">
         <v>51</v>
       </c>
@@ -10207,7 +10202,7 @@
       <c r="J19" s="89"/>
     </row>
     <row r="20" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A20" s="92"/>
+      <c r="A20" s="99"/>
       <c r="B20" s="26" t="s">
         <v>52</v>
       </c>
@@ -10235,7 +10230,7 @@
       <c r="J20" s="89"/>
     </row>
     <row r="21" spans="1:10" ht="85.5" customHeight="1">
-      <c r="A21" s="92"/>
+      <c r="A21" s="99"/>
       <c r="B21" s="26" t="s">
         <v>53</v>
       </c>
@@ -10263,7 +10258,7 @@
       <c r="J21" s="89"/>
     </row>
     <row r="22" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A22" s="92"/>
+      <c r="A22" s="99"/>
       <c r="B22" s="26" t="s">
         <v>55</v>
       </c>
@@ -10293,7 +10288,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A23" s="92"/>
+      <c r="A23" s="99"/>
       <c r="B23" s="26" t="s">
         <v>60</v>
       </c>
@@ -10323,7 +10318,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A24" s="92"/>
+      <c r="A24" s="99"/>
       <c r="B24" s="26" t="s">
         <v>195</v>
       </c>
@@ -10351,7 +10346,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A25" s="92"/>
+      <c r="A25" s="99"/>
       <c r="B25" s="26" t="s">
         <v>63</v>
       </c>
@@ -10379,7 +10374,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="31.5" customHeight="1">
-      <c r="A26" s="92"/>
+      <c r="A26" s="99"/>
       <c r="B26" s="42" t="s">
         <v>197</v>
       </c>
@@ -10407,7 +10402,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A27" s="92"/>
+      <c r="A27" s="99"/>
       <c r="B27" s="30" t="s">
         <v>66</v>
       </c>
@@ -10435,7 +10430,7 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="36.75" customHeight="1">
-      <c r="A28" s="92"/>
+      <c r="A28" s="99"/>
       <c r="B28" s="30" t="s">
         <v>68</v>
       </c>
@@ -10463,7 +10458,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="46.5" customHeight="1">
-      <c r="A29" s="92"/>
+      <c r="A29" s="99"/>
       <c r="B29" s="26" t="s">
         <v>69</v>
       </c>
@@ -10493,7 +10488,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="46.5" customHeight="1">
-      <c r="A30" s="92"/>
+      <c r="A30" s="99"/>
       <c r="B30" s="26" t="s">
         <v>72</v>
       </c>
@@ -10521,7 +10516,7 @@
       <c r="J30" s="89"/>
     </row>
     <row r="31" spans="1:10" s="58" customFormat="1" ht="66" customHeight="1">
-      <c r="A31" s="92"/>
+      <c r="A31" s="99"/>
       <c r="B31" s="42" t="s">
         <v>73</v>
       </c>
@@ -10538,7 +10533,7 @@
         <v>6005146541</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>215</v>
+        <v>154</v>
       </c>
       <c r="H31" s="59">
         <v>760</v>
@@ -10551,7 +10546,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="43.5" customHeight="1">
-      <c r="A32" s="92"/>
+      <c r="A32" s="99"/>
       <c r="B32" s="26" t="s">
         <v>74</v>
       </c>
@@ -10581,7 +10576,7 @@
       </c>
     </row>
     <row r="33" spans="1:10" ht="40.5" customHeight="1">
-      <c r="A33" s="92"/>
+      <c r="A33" s="99"/>
       <c r="B33" s="26" t="s">
         <v>77</v>
       </c>
@@ -10611,7 +10606,7 @@
       </c>
     </row>
     <row r="34" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A34" s="92"/>
+      <c r="A34" s="99"/>
       <c r="B34" s="26" t="s">
         <v>79</v>
       </c>
@@ -10641,7 +10636,7 @@
       </c>
     </row>
     <row r="35" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A35" s="92"/>
+      <c r="A35" s="99"/>
       <c r="B35" s="26" t="s">
         <v>80</v>
       </c>
@@ -10671,7 +10666,7 @@
       </c>
     </row>
     <row r="36" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A36" s="92"/>
+      <c r="A36" s="99"/>
       <c r="B36" s="26" t="s">
         <v>153</v>
       </c>
@@ -10701,7 +10696,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A37" s="92"/>
+      <c r="A37" s="99"/>
       <c r="B37" s="26" t="s">
         <v>82</v>
       </c>
@@ -10731,7 +10726,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A38" s="92"/>
+      <c r="A38" s="99"/>
       <c r="B38" s="26" t="s">
         <v>83</v>
       </c>
@@ -10761,7 +10756,7 @@
       </c>
     </row>
     <row r="39" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A39" s="92"/>
+      <c r="A39" s="99"/>
       <c r="B39" s="26" t="s">
         <v>84</v>
       </c>
@@ -10791,7 +10786,7 @@
       </c>
     </row>
     <row r="40" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A40" s="92"/>
+      <c r="A40" s="99"/>
       <c r="B40" s="26" t="s">
         <v>163</v>
       </c>
@@ -10821,7 +10816,7 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A41" s="92"/>
+      <c r="A41" s="99"/>
       <c r="B41" s="26" t="s">
         <v>85</v>
       </c>
@@ -10851,7 +10846,7 @@
       </c>
     </row>
     <row r="42" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A42" s="92"/>
+      <c r="A42" s="99"/>
       <c r="B42" s="26" t="s">
         <v>86</v>
       </c>
@@ -10881,7 +10876,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A43" s="92"/>
+      <c r="A43" s="99"/>
       <c r="B43" s="26" t="s">
         <v>88</v>
       </c>
@@ -10911,7 +10906,7 @@
       </c>
     </row>
     <row r="44" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A44" s="92"/>
+      <c r="A44" s="99"/>
       <c r="B44" s="26" t="s">
         <v>90</v>
       </c>
@@ -10941,7 +10936,7 @@
       </c>
     </row>
     <row r="45" spans="1:10" ht="39.75" customHeight="1">
-      <c r="A45" s="92"/>
+      <c r="A45" s="99"/>
       <c r="B45" s="42" t="s">
         <v>168</v>
       </c>
@@ -10971,7 +10966,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" ht="42" customHeight="1">
-      <c r="A46" s="92"/>
+      <c r="A46" s="99"/>
       <c r="B46" s="26" t="s">
         <v>173</v>
       </c>
@@ -11001,7 +10996,7 @@
       </c>
     </row>
     <row r="47" spans="1:10" ht="99.75" customHeight="1">
-      <c r="A47" s="92"/>
+      <c r="A47" s="99"/>
       <c r="B47" s="42" t="s">
         <v>174</v>
       </c>
@@ -11031,7 +11026,7 @@
       </c>
     </row>
     <row r="48" spans="1:10" ht="42" customHeight="1">
-      <c r="A48" s="92"/>
+      <c r="A48" s="99"/>
       <c r="B48" s="26" t="s">
         <v>91</v>
       </c>
@@ -11061,7 +11056,7 @@
       </c>
     </row>
     <row r="49" spans="1:10" ht="42" customHeight="1">
-      <c r="A49" s="92"/>
+      <c r="A49" s="99"/>
       <c r="B49" s="26" t="s">
         <v>92</v>
       </c>
@@ -11091,7 +11086,7 @@
       </c>
     </row>
     <row r="50" spans="1:10" ht="42" customHeight="1">
-      <c r="A50" s="92"/>
+      <c r="A50" s="99"/>
       <c r="B50" s="26" t="s">
         <v>94</v>
       </c>
@@ -11121,7 +11116,7 @@
       </c>
     </row>
     <row r="51" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A51" s="92"/>
+      <c r="A51" s="99"/>
       <c r="B51" s="26" t="s">
         <v>95</v>
       </c>
@@ -11151,7 +11146,7 @@
       </c>
     </row>
     <row r="52" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A52" s="92"/>
+      <c r="A52" s="99"/>
       <c r="B52" s="26" t="s">
         <v>96</v>
       </c>
@@ -11181,7 +11176,7 @@
       </c>
     </row>
     <row r="53" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A53" s="92"/>
+      <c r="A53" s="99"/>
       <c r="B53" s="26" t="s">
         <v>97</v>
       </c>
@@ -11211,7 +11206,7 @@
       </c>
     </row>
     <row r="54" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A54" s="92"/>
+      <c r="A54" s="99"/>
       <c r="B54" s="26" t="s">
         <v>99</v>
       </c>
@@ -11241,7 +11236,7 @@
       </c>
     </row>
     <row r="55" spans="1:10" s="58" customFormat="1" ht="85.5" customHeight="1">
-      <c r="A55" s="92"/>
+      <c r="A55" s="99"/>
       <c r="B55" s="42" t="s">
         <v>101</v>
       </c>
@@ -11271,7 +11266,7 @@
       </c>
     </row>
     <row r="56" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A56" s="92"/>
+      <c r="A56" s="99"/>
       <c r="B56" s="42" t="s">
         <v>102</v>
       </c>
@@ -11301,7 +11296,7 @@
       </c>
     </row>
     <row r="57" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A57" s="92"/>
+      <c r="A57" s="99"/>
       <c r="B57" s="42" t="s">
         <v>104</v>
       </c>
@@ -11331,7 +11326,7 @@
       </c>
     </row>
     <row r="58" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A58" s="92"/>
+      <c r="A58" s="99"/>
       <c r="B58" s="42" t="s">
         <v>105</v>
       </c>
@@ -11361,7 +11356,7 @@
       </c>
     </row>
     <row r="59" spans="1:10" s="65" customFormat="1" ht="54.75" customHeight="1">
-      <c r="A59" s="92"/>
+      <c r="A59" s="99"/>
       <c r="B59" s="56" t="s">
         <v>106</v>
       </c>
@@ -11391,7 +11386,7 @@
       </c>
     </row>
     <row r="60" spans="1:10" s="71" customFormat="1" ht="60" customHeight="1">
-      <c r="A60" s="92"/>
+      <c r="A60" s="99"/>
       <c r="B60" s="42" t="s">
         <v>210</v>
       </c>
@@ -11421,7 +11416,7 @@
       </c>
     </row>
     <row r="61" spans="1:10" ht="114" customHeight="1">
-      <c r="A61" s="92"/>
+      <c r="A61" s="99"/>
       <c r="B61" s="42" t="s">
         <v>107</v>
       </c>
@@ -11451,7 +11446,7 @@
       </c>
     </row>
     <row r="62" spans="1:10" ht="139.15" customHeight="1">
-      <c r="A62" s="92"/>
+      <c r="A62" s="99"/>
       <c r="B62" s="42" t="s">
         <v>171</v>
       </c>
@@ -11481,7 +11476,7 @@
       </c>
     </row>
     <row r="63" spans="1:10" s="58" customFormat="1" ht="93.75" customHeight="1">
-      <c r="A63" s="92"/>
+      <c r="A63" s="99"/>
       <c r="B63" s="42" t="s">
         <v>109</v>
       </c>
@@ -11511,7 +11506,7 @@
       </c>
     </row>
     <row r="64" spans="1:10" ht="135" customHeight="1">
-      <c r="A64" s="92"/>
+      <c r="A64" s="99"/>
       <c r="B64" s="42" t="s">
         <v>110</v>
       </c>
@@ -11541,7 +11536,7 @@
       </c>
     </row>
     <row r="65" spans="1:10" ht="138" customHeight="1">
-      <c r="A65" s="92"/>
+      <c r="A65" s="99"/>
       <c r="B65" s="41" t="s">
         <v>111</v>
       </c>
@@ -11571,7 +11566,7 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="96" customHeight="1">
-      <c r="A66" s="92"/>
+      <c r="A66" s="99"/>
       <c r="B66" s="41" t="s">
         <v>113</v>
       </c>
@@ -11601,7 +11596,7 @@
       </c>
     </row>
     <row r="67" spans="1:10" ht="95.25" customHeight="1">
-      <c r="A67" s="92"/>
+      <c r="A67" s="99"/>
       <c r="B67" s="42" t="s">
         <v>147</v>
       </c>
@@ -11631,7 +11626,7 @@
       </c>
     </row>
     <row r="68" spans="1:10" s="65" customFormat="1" ht="60" customHeight="1">
-      <c r="A68" s="92"/>
+      <c r="A68" s="99"/>
       <c r="B68" s="56" t="s">
         <v>116</v>
       </c>
@@ -11661,7 +11656,7 @@
       </c>
     </row>
     <row r="69" spans="1:10" ht="163.5" customHeight="1">
-      <c r="A69" s="92"/>
+      <c r="A69" s="99"/>
       <c r="B69" s="42" t="s">
         <v>117</v>
       </c>
@@ -11691,7 +11686,7 @@
       </c>
     </row>
     <row r="70" spans="1:10" ht="334.5" customHeight="1">
-      <c r="A70" s="92"/>
+      <c r="A70" s="99"/>
       <c r="B70" s="42" t="s">
         <v>119</v>
       </c>
@@ -11721,7 +11716,7 @@
       </c>
     </row>
     <row r="71" spans="1:10" s="71" customFormat="1" ht="150" customHeight="1">
-      <c r="A71" s="93"/>
+      <c r="A71" s="100"/>
       <c r="B71" s="80" t="s">
         <v>211</v>
       </c>
@@ -11849,6 +11844,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Tài liệu" ma:contentTypeID="0x010100DB24EDB465323845A68F49B67C0FBEEF" ma:contentTypeVersion="17" ma:contentTypeDescription="Tạo tài liệu mới." ma:contentTypeScope="" ma:versionID="23f0dc0ab5ad78d6e6291fdb2fe26642">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3666f02-6a17-4b93-8e4f-4f8c851bed15" xmlns:ns3="a67f3886-f84f-4ade-a9df-8a61292dc710" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c7e7713e468ce5fe561a860222c69c2e" ns2:_="" ns3:_="">
     <xsd:import namespace="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
@@ -12025,18 +12031,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64BA0B11-CE17-4EF2-86D1-BF1E203BBB04}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="a67f3886-f84f-4ade-a9df-8a61292dc710"/>
+    <ds:schemaRef ds:uri="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC0FACC-084E-4CA6-AB6A-54805DEE3D3C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC458EFE-CB2F-4B14-8A64-8A5C4D5C5CBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12053,29 +12073,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC0FACC-084E-4CA6-AB6A-54805DEE3D3C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64BA0B11-CE17-4EF2-86D1-BF1E203BBB04}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="a67f3886-f84f-4ade-a9df-8a61292dc710"/>
-    <ds:schemaRef ds:uri="c3666f02-6a17-4b93-8e4f-4f8c851bed15"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>